<commit_message>
Fix: load party (accessibilityNeeds) into trip-gen + packing controllers + add ADA filter/verify note to trip-gen prompt
- generateItinerary + generatePackingList (trips.ts) now include
  trip.party {people,pets} and user.parties[isDefault] {people,pets},
  mirroring the chat path. Previously they loaded only stops + rigs +
  travelProfile, so generateTripItineraryAI/generatePackingListAI got
  party=null and accessibilityNeeds (and all party data) was dropped
  before the prompt was built. The trip-scoped party clone already
  carried accessibilityNeeds; it was stranded by the missing include.
- generateTripItineraryAI prompt: add an ADA-filter + confirm-with-
  campground verification instruction. The note previously existed only
  in the chat/packing/modify prompts, not the initial trip-gen prompt.
- Tracker: ACCESS-1 noted DONE end-to-end through trip generation.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -3135,94 +3135,94 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="20" t="inlineStr">
         <is>
           <t>ACCESS-1</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="20" t="inlineStr">
         <is>
           <t>AccessibilityPage wired to the field the AI planner actually reads (Person.accessibilityNeeds on the user's isSelf person) instead of the ignored legacy TravelProfile.accessibilityNeeds; + best-effort disclaimer on the page; + planner 'confirm with campground' verification note</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="20" t="inlineStr">
         <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="20" t="inlineStr">
         <is>
           <t>Profile/AI</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="20" t="inlineStr">
         <is>
           <t>P1 — High</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="20" t="inlineStr">
+        <is>
+          <t>DONE end-to-end (06-04) — pending PROD verify (restart + fresh trip gen)</t>
+        </is>
+      </c>
+      <c r="G52" s="20" t="inlineStr">
+        <is>
+          <t>Yes — DB-write-path + prompt change; needs backend restart + fresh planning session</t>
+        </is>
+      </c>
+      <c r="H52" s="20" t="inlineStr">
+        <is>
+          <t>Task 2 (accessibility wiring session 06-04)</t>
+        </is>
+      </c>
+      <c r="I52" s="20" t="inlineStr">
+        <is>
+          <t>AccessibilityPage now hydrates/saves the self person's accessibilityNeeds via getDefaultParty + find-or-create-self (lazy createParty/createPerson, then updatePerson). Added isSelf to PersonCreateSchema (CREATE-only; absent from update by design — no DB uniqueness guard) so a fresh self person can be stamped. Disclaimer added above the toggles. Verify-with-campground note appended at 3 prompt sites: services/ai.ts (session planner ~L134, packing list ~L347) and controllers/ai.ts (trip-gen ~L247). Old TravelProfile.accessibilityNeeds write removed. VERIFY: needs backend restart + a NEW planning session to confirm the planner reads the self person's needs and emits the verify note. | FOLLOW-UP FIX (06-04): scout found the trip-GENERATION path dropped accessibility data — generateItinerary + generatePackingList controllers (trips.ts) loaded no party, so generateTripItineraryAI/generatePackingListAI got party=null and accessibilityNeeds never reached the prompt. FIXED: both controllers now include trip.party {people,pets} + user.parties[isDefault]{people,pets}, mirroring the chat path. Also added an ADA-filter + verify-with-campground instruction to generateTripItineraryAI prompt (the note had only been in chat/packing/modify prompts, not initial trip-gen). Wiring is now complete END-TO-END through trip generation. VERIFY: needs backend restart + a FRESH trip generation on PROD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="20" t="inlineStr">
+        <is>
+          <t>PROFILE-PHONE-1</t>
+        </is>
+      </c>
+      <c r="B53" s="20" t="inlineStr">
+        <is>
+          <t>Hide unused Phone field on ProfilePage (hide-not-drop)</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>Bug/Polish</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="E53" s="20" t="inlineStr">
+        <is>
+          <t>P3 — Low / cosmetic</t>
+        </is>
+      </c>
+      <c r="F53" s="20" t="inlineStr">
         <is>
           <t>DONE (06-04) — pending PROD verify</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Yes — DB-write-path + prompt change; needs backend restart + fresh planning session</t>
-        </is>
-      </c>
-      <c r="H52" t="inlineStr">
+      <c r="G53" s="20" t="inlineStr">
+        <is>
+          <t>Yes — UI-only; confirm field gone + stored values intact</t>
+        </is>
+      </c>
+      <c r="H53" s="20" t="inlineStr">
         <is>
           <t>Task 2 (accessibility wiring session 06-04)</t>
         </is>
       </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>AccessibilityPage now hydrates/saves the self person's accessibilityNeeds via getDefaultParty + find-or-create-self (lazy createParty/createPerson, then updatePerson). Added isSelf to PersonCreateSchema (CREATE-only; absent from update by design — no DB uniqueness guard) so a fresh self person can be stamped. Disclaimer added above the toggles. Verify-with-campground note appended at 3 prompt sites: services/ai.ts (session planner ~L134, packing list ~L347) and controllers/ai.ts (trip-gen ~L247). Old TravelProfile.accessibilityNeeds write removed. VERIFY: needs backend restart + a NEW planning session to confirm the planner reads the self person's needs and emits the verify note.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>PROFILE-PHONE-1</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Hide unused Phone field on ProfilePage (hide-not-drop)</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Bug/Polish</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Profile</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>P3 — Low / cosmetic</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>DONE (06-04) — pending PROD verify</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Yes — UI-only; confirm field gone + stored values intact</t>
-        </is>
-      </c>
-      <c r="H53" t="inlineStr">
-        <is>
-          <t>Task 2 (accessibility wiring session 06-04)</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
+      <c r="I53" s="20" t="inlineStr">
         <is>
           <t>Removed only the Phone &lt;div&gt; (label + type=tel input) from ProfilePage.tsx. register('phone') default, Prisma User.phone column, server handler, and User.phone TS type all left untouched so any stored values persist. No other live reference to phone remains in ProfilePage. Verify in browser.</t>
         </is>

</xml_diff>

<commit_message>
UX-HOME-PREFILL: pre-fill save-home modal with full address via optional startAddress in itinerary contract
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -3319,6 +3319,53 @@
       <c r="I55" s="20" t="inlineStr">
         <is>
           <t>Scout finding while fixing ACCESS-1. The defaultParty.people.map clone in createTrip copies role, name, age, isTraveling, isEmergencyContact, emergencyPhone, accessibilityNeeds, dietaryNotes, militaryStatus, firstResponder — but NOT isSelf (added in the prior schema task). So a trip-scoped clone has no self person. Harmless today (accessibility is aggregated across all traveling people, not just self), but any future trip-scoped self lookup would fail. Add isSelf: p.isSelf to the clone map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="20" t="inlineStr">
+        <is>
+          <t>UX-HOME-PREFILL</t>
+        </is>
+      </c>
+      <c r="B56" s="20" t="inlineStr">
+        <is>
+          <t>Save-home ("Starting from") modal pre-fills only city/state, not the full street address the user typed in chat</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>Bug/Polish</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="inlineStr">
+        <is>
+          <t>Trips/AI</t>
+        </is>
+      </c>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>P3 — Low / convenience</t>
+        </is>
+      </c>
+      <c r="F56" s="20" t="inlineStr">
+        <is>
+          <t>DONE (06-04) — pending PROD verify</t>
+        </is>
+      </c>
+      <c r="G56" s="20" t="inlineStr">
+        <is>
+          <t>Yes — AI-contract + prompt change; needs backend restart + a FRESH no-home planning session (address only flows through on a newly planned trip)</t>
+        </is>
+      </c>
+      <c r="H56" s="20" t="inlineStr">
+        <is>
+          <t>UX-HOME-PREFILL task (session 06-04)</t>
+        </is>
+      </c>
+      <c r="I56" s="20" t="inlineStr">
+        <is>
+          <t>Root cause was upstream at the AI layer: the HOME stop in the &lt;itinerary&gt; JSON contract carried only locationName/locationState (city/ST), so the user’s full typed address ("1234 Example St, Mesa, AZ 85201") was reduced to "Mesa, AZ" before any structured data reached the client; SessionPage built the modal pre-fill as [city, ST].join. FIX (additive only): added an OPTIONAL startAddress string to the HOME stop in the AI contract (services/ai.ts — instruction ~L118 + JSON example ~L202) instructing the model to copy the user’s VERBATIM starting-location text into startAddress ONLY when they typed a full street address, keeping locationName/locationState as city/ST for planning (unchanged); added optional startAddress?: string to the client Stop type (types/index.ts); SessionPage buildItinerary now pre-fills address: startStop?.startAddress || [city, ST].join (falls back to City, ST). SAVE path untouched — modal still requires a Google Places re-pick (8-field write). Server createStop whitelists fields so startAddress is never persisted. Client build green; server tsc clean (only pre-existing junction-path artifacts in redis.ts/prisma.ts). VERIFY: restart backend + plan a NEW no-home trip with a full typed street address → the “Starting from…” modal title + AddressAutocomplete seed should show the full address.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix AI-MESA-4: forbid inventing origin when user says 'you pick' (no-home)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -3366,6 +3366,53 @@
       <c r="I56" s="20" t="inlineStr">
         <is>
           <t>Root cause was upstream at the AI layer: the HOME stop in the &lt;itinerary&gt; JSON contract carried only locationName/locationState (city/ST), so the user’s full typed address ("1234 Example St, Mesa, AZ 85201") was reduced to "Mesa, AZ" before any structured data reached the client; SessionPage built the modal pre-fill as [city, ST].join. FIX (additive only): added an OPTIONAL startAddress string to the HOME stop in the AI contract (services/ai.ts — instruction ~L118 + JSON example ~L202) instructing the model to copy the user’s VERBATIM starting-location text into startAddress ONLY when they typed a full street address, keeping locationName/locationState as city/ST for planning (unchanged); added optional startAddress?: string to the client Stop type (types/index.ts); SessionPage buildItinerary now pre-fills address: startStop?.startAddress || [city, ST].join (falls back to City, ST). SAVE path untouched — modal still requires a Google Places re-pick (8-field write). Server createStop whitelists fields so startAddress is never persisted. Client build green; server tsc clean (only pre-existing junction-path artifacts in redis.ts/prisma.ts). VERIFY: restart backend + plan a NEW no-home trip with a full typed street address → the “Starting from…” modal title + AddressAutocomplete seed should show the full address.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="20" t="inlineStr">
+        <is>
+          <t>AI-MESA-4</t>
+        </is>
+      </c>
+      <c r="B57" s="20" t="inlineStr">
+        <is>
+          <t>No-home user who asks the AI to PICK their starting point gets a fabricated home city ("...from my home address you pick" / "you pick" applied to the ORIGIN → planner invents an origin city)</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="D57" s="20" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="E57" s="20" t="inlineStr">
+        <is>
+          <t>P1 — High</t>
+        </is>
+      </c>
+      <c r="F57" s="20" t="inlineStr">
+        <is>
+          <t>DONE (06-04) — pending PROD verify</t>
+        </is>
+      </c>
+      <c r="G57" s="20" t="inlineStr">
+        <is>
+          <t>Yes — prompt/service-only; needs backend restart + a FRESH no-home planning session</t>
+        </is>
+      </c>
+      <c r="H57" s="20" t="inlineStr">
+        <is>
+          <t>scout 06-04 (AI-MESA-4 task)</t>
+        </is>
+      </c>
+      <c r="I57" s="20" t="inlineStr">
+        <is>
+          <t>Same family as AI-MESA-1/2/3. REPRO: no-home user (all home fields NULL) sent "the 3-day trip to Sedona starting from my home address you pick, leave this Saturday" → planner replied "I will use your home address in Billings as the starting point" (Billings INVENTED). DISTINCTION: AI-MESA-3 closed the case where the user merely SAYS "home"; AI-MESA-4 is when the user affirmatively asks the AI to CHOOSE/supply the origin ("you pick", "pick a home for me"). ROOT CAUSE (scout): the AI-MESA-3 noHomeDirective (services/ai.ts ~L87, injected only when !homeCity &amp;&amp; !homeLocation) enumerated trigger phrases ("home"/"my home"/"from home"/"use my home address") but NOT the "you pick"/"choose a starting point" angle; meanwhile the Surprise-trip rule (~L107) lists "you pick" as a license to defer the DESTINATION choice to the AI, with no carve-out that deferral must NOT extend to the origin. The model conflated picking a destination with picking a home and fabricated Billings. The static NO HOME ON FILE rule (~L176) is gated on "user names no starting location," which a model can treat as not firing once "you pick" is read as a start instruction. FIX (PRIMARY only, additive, +1/-1 in services/ai.ts:87): extended the existing noHomeDirective string to add — "This includes when the user asks YOU to choose or supply the starting point — e.g. you pick, pick a home for me, choose a starting point, from my home address you pick, or any request that you select/guess/invent the origin. Deferring the DESTINATION choice to you (a surprise trip) NEVER extends to the starting location: you may choose where they GO, but you must NEVER choose, invent, or assume where they START FROM." No-home-scoped (zero effect on home-on-file users — hasHomeOnFile branch byte-for-byte unchanged) and zero effect on destination surprise trips. Secondary surprise-trip edit (~L107) intentionally NOT applied (smaller blast radius preferred). Grep check: no real city name in the no-home/origin directive (only placeholders + forbidden-behavior text). Client tsc+vite green; server tsc clean for ai.ts (only pre-existing redis.ts/prisma.ts TS2742 junction artifacts). VERIFY: restart backend + fresh no-home session; "to Sedona starting from my home address you pick" must ASK "Where will you be starting from?" and name NO city, while a genuine destination "you pick / surprise me" still picks a destination.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix AI-MESA-5: no-home user with destination-only must be asked for origin, never fabricate
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I57"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -3413,6 +3413,53 @@
       <c r="I57" s="20" t="inlineStr">
         <is>
           <t>Same family as AI-MESA-1/2/3. REPRO: no-home user (all home fields NULL) sent "the 3-day trip to Sedona starting from my home address you pick, leave this Saturday" → planner replied "I will use your home address in Billings as the starting point" (Billings INVENTED). DISTINCTION: AI-MESA-3 closed the case where the user merely SAYS "home"; AI-MESA-4 is when the user affirmatively asks the AI to CHOOSE/supply the origin ("you pick", "pick a home for me"). ROOT CAUSE (scout): the AI-MESA-3 noHomeDirective (services/ai.ts ~L87, injected only when !homeCity &amp;&amp; !homeLocation) enumerated trigger phrases ("home"/"my home"/"from home"/"use my home address") but NOT the "you pick"/"choose a starting point" angle; meanwhile the Surprise-trip rule (~L107) lists "you pick" as a license to defer the DESTINATION choice to the AI, with no carve-out that deferral must NOT extend to the origin. The model conflated picking a destination with picking a home and fabricated Billings. The static NO HOME ON FILE rule (~L176) is gated on "user names no starting location," which a model can treat as not firing once "you pick" is read as a start instruction. FIX (PRIMARY only, additive, +1/-1 in services/ai.ts:87): extended the existing noHomeDirective string to add — "This includes when the user asks YOU to choose or supply the starting point — e.g. you pick, pick a home for me, choose a starting point, from my home address you pick, or any request that you select/guess/invent the origin. Deferring the DESTINATION choice to you (a surprise trip) NEVER extends to the starting location: you may choose where they GO, but you must NEVER choose, invent, or assume where they START FROM." No-home-scoped (zero effect on home-on-file users — hasHomeOnFile branch byte-for-byte unchanged) and zero effect on destination surprise trips. Secondary surprise-trip edit (~L107) intentionally NOT applied (smaller blast radius preferred). Grep check: no real city name in the no-home/origin directive (only placeholders + forbidden-behavior text). Client tsc+vite green; server tsc clean for ai.ts (only pre-existing redis.ts/prisma.ts TS2742 junction artifacts). VERIFY: restart backend + fresh no-home session; "to Sedona starting from my home address you pick" must ASK "Where will you be starting from?" and name NO city, while a genuine destination "you pick / surprise me" still picks a destination.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="20" t="inlineStr">
+        <is>
+          <t>AI-MESA-5</t>
+        </is>
+      </c>
+      <c r="B58" s="20" t="inlineStr">
+        <is>
+          <t>No-home user who names a DESTINATION but no origin (and no trigger words) gets a fabricated starting city — nondeterministic hallucination (run 1 "Austin", run 2 "Boerne, TX")</t>
+        </is>
+      </c>
+      <c r="C58" s="20" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>P1 — High</t>
+        </is>
+      </c>
+      <c r="F58" s="20" t="inlineStr">
+        <is>
+          <t>DONE (06-04) — pending PROD verify</t>
+        </is>
+      </c>
+      <c r="G58" s="20" t="inlineStr">
+        <is>
+          <t>Yes — prompt/service-only; needs backend restart + a FRESH no-home planning session</t>
+        </is>
+      </c>
+      <c r="H58" s="20" t="inlineStr">
+        <is>
+          <t>scout 06-04 (AI-MESA-5 task)</t>
+        </is>
+      </c>
+      <c r="I58" s="20" t="inlineStr">
+        <is>
+          <t>Fourth in the no-home phantom-origin family (AI-MESA-1/2/3/4). DISTINCT from all priors: NO trigger words at all — user did NOT say "home" (MESA-3) and did NOT say "you pick" (MESA-4). REPRO: no-home user (all home fields NULL, confirmed empty) typed "start a trip to sedona starting tomorrow for 3 days" — named a DESTINATION + date + duration, but NO origin. On TWO fresh sessions the planner invented a DIFFERENT origin each run: run 1 "I will use your home address in Austin", run 2 "starting from Boerne, TX". Nondeterministic (different invented TX city each run, nothing stored) =&gt; pure hallucination, not stored-data read. GATE WAS CORRECT: controller sets homeCity/homeState/homeLocation -&gt; undefined when NULL (controllers/ai.ts ~500-503), so hasHomeOnFile=!!(undefined||undefined)=false and the noHomeDirective IS injected (services/ai.ts 84-93). The model was OVERRIDING a present directive. TWO REINFORCING ROOT CAUSES (scout): (1) the JSON itinerary contract (~L118) requires an order-1 HOME stop "regardless of whether the user mentioned it explicitly" — once the model has destination+dates it rushes to emit &lt;itinerary&gt; and the mandatory HOME stop FORCES an origin city, which it fabricates; (2) the HOME ON FILE template (~L177) has a second trigger "OR if the user mentions no starting location at all" with an open [CITY] slot — that trigger matches this exact input, and run 1 output is that template verbatim with [CITY] hallucinated. Neither the noHomeDirective nor the static NO HOME ON FILE rule (~L176) said a named destination does NOT substitute for an origin, nor that you must not emit an itinerary / fill the HOME stop without a real origin. FIX (additive only, BOTH blocks land INSIDE the no-home-scoped noHomeDirective string at services/ai.ts:87, +1/-1; zero effect on home-on-file users since the hasHomeOnFile "" branch is byte-for-byte unchanged; did NOT touch L118/L176/L177/L107 or any JSON field): (a) "A named DESTINATION is NOT a starting location... a destination, dates, and duration do NOT give you enough to begin planning... Until the user gives a real starting city, do NOT emit an &lt;itinerary&gt; block and do NOT populate the order-1 HOME stop with any city; the origin must be the user own typed words, never a value you generate." (b) "Never output the sentence I will use your home address in [city] or fill any home-address or [CITY] slot for this user — that line is reserved exclusively for users with a real saved home, which this user does not have." Block (a) removes the destination-is-enough loophole + HOME-stop pressure; block (b) disarms the exact template the model used to fabricate Austin. Grep check: no real place name in the noHomeDirective string (only placeholders "some destination", [city], [CITY]). Client tsc+vite green; server tsc clean for ai.ts (only pre-existing redis.ts/prisma.ts TS2742 junction artifacts). VERIFY: restart backend + fresh no-home session; "trip to &lt;dest&gt; starting tomorrow for 3 days" must ASK "Where will you be starting from?" and name NO city + emit NO itinerary until the user gives an origin; genuine named-origin and surprise-destination flows must still work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix AI-MESA-6: replace hardcoded example cities in prompt with placeholders (stop model copying them as origin)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -3460,6 +3460,53 @@
       <c r="I58" s="20" t="inlineStr">
         <is>
           <t>Fourth in the no-home phantom-origin family (AI-MESA-1/2/3/4). DISTINCT from all priors: NO trigger words at all — user did NOT say "home" (MESA-3) and did NOT say "you pick" (MESA-4). REPRO: no-home user (all home fields NULL, confirmed empty) typed "start a trip to sedona starting tomorrow for 3 days" — named a DESTINATION + date + duration, but NO origin. On TWO fresh sessions the planner invented a DIFFERENT origin each run: run 1 "I will use your home address in Austin", run 2 "starting from Boerne, TX". Nondeterministic (different invented TX city each run, nothing stored) =&gt; pure hallucination, not stored-data read. GATE WAS CORRECT: controller sets homeCity/homeState/homeLocation -&gt; undefined when NULL (controllers/ai.ts ~500-503), so hasHomeOnFile=!!(undefined||undefined)=false and the noHomeDirective IS injected (services/ai.ts 84-93). The model was OVERRIDING a present directive. TWO REINFORCING ROOT CAUSES (scout): (1) the JSON itinerary contract (~L118) requires an order-1 HOME stop "regardless of whether the user mentioned it explicitly" — once the model has destination+dates it rushes to emit &lt;itinerary&gt; and the mandatory HOME stop FORCES an origin city, which it fabricates; (2) the HOME ON FILE template (~L177) has a second trigger "OR if the user mentions no starting location at all" with an open [CITY] slot — that trigger matches this exact input, and run 1 output is that template verbatim with [CITY] hallucinated. Neither the noHomeDirective nor the static NO HOME ON FILE rule (~L176) said a named destination does NOT substitute for an origin, nor that you must not emit an itinerary / fill the HOME stop without a real origin. FIX (additive only, BOTH blocks land INSIDE the no-home-scoped noHomeDirective string at services/ai.ts:87, +1/-1; zero effect on home-on-file users since the hasHomeOnFile "" branch is byte-for-byte unchanged; did NOT touch L118/L176/L177/L107 or any JSON field): (a) "A named DESTINATION is NOT a starting location... a destination, dates, and duration do NOT give you enough to begin planning... Until the user gives a real starting city, do NOT emit an &lt;itinerary&gt; block and do NOT populate the order-1 HOME stop with any city; the origin must be the user own typed words, never a value you generate." (b) "Never output the sentence I will use your home address in [city] or fill any home-address or [CITY] slot for this user — that line is reserved exclusively for users with a real saved home, which this user does not have." Block (a) removes the destination-is-enough loophole + HOME-stop pressure; block (b) disarms the exact template the model used to fabricate Austin. Grep check: no real place name in the noHomeDirective string (only placeholders "some destination", [city], [CITY]). Client tsc+vite green; server tsc clean for ai.ts (only pre-existing redis.ts/prisma.ts TS2742 junction artifacts). VERIFY: restart backend + fresh no-home session; "trip to &lt;dest&gt; starting tomorrow for 3 days" must ASK "Where will you be starting from?" and name NO city + emit NO itinerary until the user gives an origin; genuine named-origin and surprise-destination flows must still work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="20" t="inlineStr">
+        <is>
+          <t>AI-MESA-6</t>
+        </is>
+      </c>
+      <c r="B59" s="20" t="inlineStr">
+        <is>
+          <t>Hardcoded REAL example cities in the planning prompt get COPIED by the model to fill the order-1 HOME stop for no-home users (borrowed "Lubbock" from the itinerary-contract transit example; same class as the earlier "Fargo" borrow)</t>
+        </is>
+      </c>
+      <c r="C59" s="20" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="E59" s="20" t="inlineStr">
+        <is>
+          <t>P1 — High</t>
+        </is>
+      </c>
+      <c r="F59" s="20" t="inlineStr">
+        <is>
+          <t>DONE (06-04) — pending PROD verify</t>
+        </is>
+      </c>
+      <c r="G59" s="20" t="inlineStr">
+        <is>
+          <t>Yes — prompt-only; needs backend restart + a FRESH no-home planning session</t>
+        </is>
+      </c>
+      <c r="H59" s="20" t="inlineStr">
+        <is>
+          <t>scout 06-04 (AI-MESA-6 task)</t>
+        </is>
+      </c>
+      <c r="I59" s="20" t="inlineStr">
+        <is>
+          <t>Fifth in the no-home phantom-origin family. ROOT CAUSE: EXAMPLE-BORROWING — same class as AI-MESA-2 (model copied "Fargo" from a prompt origin example). DB scout proved prod momann has ALL home fields NULL (incl. homeState), so it was not a data leak; the model was lifting a concrete city PRINTED IN THE PROMPT EXAMPLES to satisfy the mandatory order-1 HOME stop. The deterministic "Lubbock" (vs MESA-5 wandering hallucination) was the tell: Lubbock was the hardcoded OVERNIGHT_ONLY transit-stop in the &lt;itinerary&gt; JSON contract example (services/ai.ts:215/219). The MESA-5 noHomeDirective cannot beat a real city literally shown as data to copy. FIX (prompt-only, additive-safe, +12/-12 in services/ai.ts; NO logic / noHomeDirective / hasHomeOnFile / HOME-stop instruction / JSON keys/structure changed): replaced EVERY real place name in EXAMPLE/TEMPLATE/JSON-contract content of the planning-chat prompt with unmistakable bracketed ALL-CAPS placeholders the model cannot mistake for copyable data. Full sweep: L159 Del Rio/Flagstaff -&gt; [EXAMPLE_DESTINATION]; L163 Williams/Sedona -&gt; [EXAMPLE_STOP_1]/[EXAMPLE_STOP_2]; L166 Prada Marfa/Marfa/Marfa Lights -&gt; [EXAMPLE_POI]; L180 campground samples -&gt; [EXAMPLE_CAMPGROUND_1..3]; L186 Denver/Moab -&gt; [EXAMPLE_DESTINATION_A]/[EXAMPLE_DESTINATION_B]; L188 Albuquerque -&gt; [EXAMPLE_DESTINATION]; JSON example L215/216 Lubbock/TX -&gt; [EXAMPLE_TRANSIT_CITY]/[STATE], L219 transit campgrounds -&gt; placeholders, L229/230 Albuquerque/NM -&gt; [EXAMPLE_DESTINATION_CITY]/[STATE], L233 dest campgrounds -&gt; placeholders. JSON example re-validated: parses, 3 stops, identical 13 keys per stop, only string VALUES changed. FLAGGED + LEFT UNCHANGED (genuine RULE data, not copyable itinerary examples): L153 towing-hazard roads (Big Sur/CA-1, Tail of the Dragon US-129, Going-to-the-Sun/Glacier NP — roads to AVOID); L154 truck-stop brands (Pilot/Flying J/Love's/TA/Petro — fuel rule); L156 NV/UT/WY (long-stretch fuel guidance). Other prompts (generateTripItineraryAI/highway helper L472/562/563) use highway designations only (no city names — prompt forbids them), out of scope. Grep check: only place names remaining in the planning prompt are bracketed placeholders + the 3 flagged genuine-rule sets. Client tsc+vite green; server tsc clean for ai.ts (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). VERIFY: restart backend + fresh no-home session; "trip to &lt;dest&gt;" with no origin must ASK "Where will you be starting from?" and must NOT emit Lubbock/any example city as the HOME stop. KEY LESSON (recurring): ANY real place name printed in a prompt example is copyable data to the model; every example city must be a placeholder. Future ai.ts prompt edits must end with a grep that all example origins/stops/campgrounds are bracketed placeholders.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AI-MESA-7: tracker row (deterministic origin guard)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I59"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -3507,6 +3507,53 @@
       <c r="I59" s="20" t="inlineStr">
         <is>
           <t>Fifth in the no-home phantom-origin family. ROOT CAUSE: EXAMPLE-BORROWING — same class as AI-MESA-2 (model copied "Fargo" from a prompt origin example). DB scout proved prod momann has ALL home fields NULL (incl. homeState), so it was not a data leak; the model was lifting a concrete city PRINTED IN THE PROMPT EXAMPLES to satisfy the mandatory order-1 HOME stop. The deterministic "Lubbock" (vs MESA-5 wandering hallucination) was the tell: Lubbock was the hardcoded OVERNIGHT_ONLY transit-stop in the &lt;itinerary&gt; JSON contract example (services/ai.ts:215/219). The MESA-5 noHomeDirective cannot beat a real city literally shown as data to copy. FIX (prompt-only, additive-safe, +12/-12 in services/ai.ts; NO logic / noHomeDirective / hasHomeOnFile / HOME-stop instruction / JSON keys/structure changed): replaced EVERY real place name in EXAMPLE/TEMPLATE/JSON-contract content of the planning-chat prompt with unmistakable bracketed ALL-CAPS placeholders the model cannot mistake for copyable data. Full sweep: L159 Del Rio/Flagstaff -&gt; [EXAMPLE_DESTINATION]; L163 Williams/Sedona -&gt; [EXAMPLE_STOP_1]/[EXAMPLE_STOP_2]; L166 Prada Marfa/Marfa/Marfa Lights -&gt; [EXAMPLE_POI]; L180 campground samples -&gt; [EXAMPLE_CAMPGROUND_1..3]; L186 Denver/Moab -&gt; [EXAMPLE_DESTINATION_A]/[EXAMPLE_DESTINATION_B]; L188 Albuquerque -&gt; [EXAMPLE_DESTINATION]; JSON example L215/216 Lubbock/TX -&gt; [EXAMPLE_TRANSIT_CITY]/[STATE], L219 transit campgrounds -&gt; placeholders, L229/230 Albuquerque/NM -&gt; [EXAMPLE_DESTINATION_CITY]/[STATE], L233 dest campgrounds -&gt; placeholders. JSON example re-validated: parses, 3 stops, identical 13 keys per stop, only string VALUES changed. FLAGGED + LEFT UNCHANGED (genuine RULE data, not copyable itinerary examples): L153 towing-hazard roads (Big Sur/CA-1, Tail of the Dragon US-129, Going-to-the-Sun/Glacier NP — roads to AVOID); L154 truck-stop brands (Pilot/Flying J/Love's/TA/Petro — fuel rule); L156 NV/UT/WY (long-stretch fuel guidance). Other prompts (generateTripItineraryAI/highway helper L472/562/563) use highway designations only (no city names — prompt forbids them), out of scope. Grep check: only place names remaining in the planning prompt are bracketed placeholders + the 3 flagged genuine-rule sets. Client tsc+vite green; server tsc clean for ai.ts (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). VERIFY: restart backend + fresh no-home session; "trip to &lt;dest&gt;" with no origin must ASK "Where will you be starting from?" and must NOT emit Lubbock/any example city as the HOME stop. KEY LESSON (recurring): ANY real place name printed in a prompt example is copyable data to the model; every example city must be a placeholder. Future ai.ts prompt edits must end with a grep that all example origins/stops/campgrounds are bracketed placeholders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="20" t="inlineStr">
+        <is>
+          <t>AI-MESA-7</t>
+        </is>
+      </c>
+      <c r="B60" s="20" t="inlineStr">
+        <is>
+          <t>Deterministic server-side origin guard — block fabricated HOME city for no-home users (prompt fixes MESA-4/5/6 proven insufficient: 7 runs, 6 fabricated origins)</t>
+        </is>
+      </c>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>Bug/Hardening</t>
+        </is>
+      </c>
+      <c r="D60" s="20" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="F60" s="20" t="inlineStr">
+        <is>
+          <t>DONE (06-04) - pending PROD verify</t>
+        </is>
+      </c>
+      <c r="G60" s="20" t="inlineStr">
+        <is>
+          <t>Yes - server post-generation guard; needs backend restart + fresh no-home session</t>
+        </is>
+      </c>
+      <c r="H60" s="20" t="inlineStr">
+        <is>
+          <t>scout 06-04 (AI-MESA-7 task)</t>
+        </is>
+      </c>
+      <c r="I60" s="20" t="inlineStr">
+        <is>
+          <t>Hardening fix: prompt-level fixes (AI-MESA-4/5/6) were PROVEN insufficient to stop origin fabrication for no-home users — destination-only prompts, 7 runs, only 1 correctly asked 'Where will you be starting from?'; the other 6 invented different origins (Los Angeles, Bullhead City x2, Grand Junction, Pinecrest-as-origin). The model invents an origin to satisfy the mandatory order-1 HOME stop; its compliance cannot be relied on. FIX = DETERMINISTIC server-side guard (Option A from scout), additive only in controllers/ai.ts (+92/-0), no prompt / services/ai.ts / JSON-contract change. Flow: planning is ONE generation (chatWithAI ~:598) with &lt;itinerary&gt; embedded in the reply; the server never parsed it before (client parseItinerary did). Added: (1) NO_ORIGIN_RESPONSE canned constant beside HARD_CAP_RESPONSE — contains NO &lt;itinerary&gt;, so the client shows no Build button; (2) parseItineraryBlock(text) helper mirroring the client parser (regex extract + JSON.parse, try/catch, returns null on miss/parse-fail, never throws =&gt; fails OPEN); (3) guard inserted AFTER generation + AFTER the modify-retry block, BEFORE persist + res.json, so it mutates response in time and the canned ask (not the bogus itinerary) is what gets persisted/returned. DETECTION: hasHomeOnFile = !!(userProfile.homeCity || userProfile.homeLocation); only if context !== 'modify' AND !hasHomeOnFile; parse the itinerary; if stops[0].type === 'HOME', normalize (lowercase, strip non-alphanumeric to spaces) the HOME city and ALL user-role message text; if the city is non-empty AND appears in NONE of the user messages =&gt; fabricated =&gt; response = NO_ORIGIN_RESPONSE + console.warn the blocked city/state for observability. FALSE-POSITIVE GUARDS (conservative — they only WIDEN what counts as user-provided, so they can only REDUCE false positives and never let a fabricated city through): also treat the origin as user-provided if the user typed the verbatim startAddress the model copied, or typed BOTH the city AND its state (state alone never counts). BLAST RADIUS: fires ONLY for no-home + planning + parseable HOME-stop itinerary + city-never-typed. Home-on-file users (hasHomeOnFile true), modify mode (context gate), non-itinerary turns (parse null), and user-typed-origin (substring match) are ALL untouched. Worst case is a phrasing mismatch =&gt; user re-asked once (their re-answer contains the city verbatim =&gt; builds next turn); NEVER a broken trip or data loss. This is the code-level guarantee behind the MESA-4/5/6 prompt nudges. Client tsc+vite green; server tsc clean for the guard (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). VERIFY: restart backend + fresh no-home session; a destination-only prompt must return the canned ask and NO Build button across repeated runs (deterministic), while named-origin and home-on-file flows build normally and modify mode is unaffected.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix AI-MESA-9: forbid origin-assertion in prompt for no-home users + fix prose-guard regex hole
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -3554,6 +3554,53 @@
       <c r="I60" s="20" t="inlineStr">
         <is>
           <t>Hardening fix: prompt-level fixes (AI-MESA-4/5/6) were PROVEN insufficient to stop origin fabrication for no-home users — destination-only prompts, 7 runs, only 1 correctly asked 'Where will you be starting from?'; the other 6 invented different origins (Los Angeles, Bullhead City x2, Grand Junction, Pinecrest-as-origin). The model invents an origin to satisfy the mandatory order-1 HOME stop; its compliance cannot be relied on. FIX = DETERMINISTIC server-side guard (Option A from scout), additive only in controllers/ai.ts (+92/-0), no prompt / services/ai.ts / JSON-contract change. Flow: planning is ONE generation (chatWithAI ~:598) with &lt;itinerary&gt; embedded in the reply; the server never parsed it before (client parseItinerary did). Added: (1) NO_ORIGIN_RESPONSE canned constant beside HARD_CAP_RESPONSE — contains NO &lt;itinerary&gt;, so the client shows no Build button; (2) parseItineraryBlock(text) helper mirroring the client parser (regex extract + JSON.parse, try/catch, returns null on miss/parse-fail, never throws =&gt; fails OPEN); (3) guard inserted AFTER generation + AFTER the modify-retry block, BEFORE persist + res.json, so it mutates response in time and the canned ask (not the bogus itinerary) is what gets persisted/returned. DETECTION: hasHomeOnFile = !!(userProfile.homeCity || userProfile.homeLocation); only if context !== 'modify' AND !hasHomeOnFile; parse the itinerary; if stops[0].type === 'HOME', normalize (lowercase, strip non-alphanumeric to spaces) the HOME city and ALL user-role message text; if the city is non-empty AND appears in NONE of the user messages =&gt; fabricated =&gt; response = NO_ORIGIN_RESPONSE + console.warn the blocked city/state for observability. FALSE-POSITIVE GUARDS (conservative — they only WIDEN what counts as user-provided, so they can only REDUCE false positives and never let a fabricated city through): also treat the origin as user-provided if the user typed the verbatim startAddress the model copied, or typed BOTH the city AND its state (state alone never counts). BLAST RADIUS: fires ONLY for no-home + planning + parseable HOME-stop itinerary + city-never-typed. Home-on-file users (hasHomeOnFile true), modify mode (context gate), non-itinerary turns (parse null), and user-typed-origin (substring match) are ALL untouched. Worst case is a phrasing mismatch =&gt; user re-asked once (their re-answer contains the city verbatim =&gt; builds next turn); NEVER a broken trip or data loss. This is the code-level guarantee behind the MESA-4/5/6 prompt nudges. Client tsc+vite green; server tsc clean for the guard (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). VERIFY: restart backend + fresh no-home session; a destination-only prompt must return the canned ask and NO Build button across repeated runs (deterministic), while named-origin and home-on-file flows build normally and modify mode is unaffected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="20" t="inlineStr">
+        <is>
+          <t>AI-MESA-9</t>
+        </is>
+      </c>
+      <c r="B61" s="20" t="inlineStr">
+        <is>
+          <t>Close no-home origin fabrication at the SOURCE (prompt forbids origin assertion when no origin exists) + build the prose-assertion guard with hole-free regex (home address in Phoenix slipped) - layered with MESA-7 itinerary guard</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>Bug/Hardening</t>
+        </is>
+      </c>
+      <c r="D61" s="20" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="E61" s="20" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="F61" s="20" t="inlineStr">
+        <is>
+          <t>DONE (06-04) - pending PROD verify</t>
+        </is>
+      </c>
+      <c r="G61" s="20" t="inlineStr">
+        <is>
+          <t>Yes - prompt + server guard; needs backend restart + fresh no-home session</t>
+        </is>
+      </c>
+      <c r="H61" s="20" t="inlineStr">
+        <is>
+          <t>AI-MESA-9 task 06-04</t>
+        </is>
+      </c>
+      <c r="I61" s="20" t="inlineStr">
+        <is>
+          <t>Belt-and-suspenders close of the no-home origin-fabrication category. Two prior leaks proved single-layer fixes insufficient: (i) prompt nudges (MESA-4/5/6) do not reliably stop the model naming a fabricated origin; (ii) the MESA-7 deterministic guard only inspects the &lt;itinerary&gt; JSON, so a fabricated origin stated only in PRE-ITINERARY PROSE slipped (prompt 'trip to Pittsburgh' -&gt; assistant 'Got it - starting from Columbus, Ohio', not blocked; and 'home address in Phoenix' style phrasings). NOTE: the MESA-8 prose-guard was SCOUTED earlier but never built - this task built it correctly from the start (no pre-existing extractAssertedOrigin existed on main). THREE additive changes: CHANGE 1 (PROMPT, services/ai.ts ~175-176): made the origin-naming confirmation templates EXPLICITLY CONDITIONAL and added a HARD RULE right where they are defined - the 'starting from [City, State]' and 'I'll use your home address in [CITY]' lines may be used ONLY when a real origin exists (user typed a starting city/address OR a real home is on file). When NO home on file AND no typed origin, the model is FORBIDDEN to emit any sentence naming a starting city and the ONLY permitted origin response is to ask 'Where will you be starting from?'. Placeholders only (per MESA-6 lesson); grep-verified no real city names added. No change to JSON contract / order-1 HOME instruction / noHomeDirective / hasHomeOnFile. CHANGE 2 (controllers/ai.ts): added extractAssertedOrigin(text) - an ORIGIN-ANCHORED prose scanner that returns the asserted city's first proper-noun token (single-token capture) or null, and a sibling guard block inside the existing MESA-7 no-home gate (computes its own norm/userText so the MESA-7 block is left byte-for-byte unchanged): if a no-home user's reply asserts a starting city whose first token appears in NONE of the user messages, response is replaced with NO_ORIGIN_RESPONSE. Anchors cover the scripted templates plus widened phrasings: starting from X, home address/base in|is X, your home in|is X, X as the starting point, leaving/departing (from) X, set off from X, kick off in X, launch point is X, starting point is X, begin in X. Uppercase-first-letter + stopword (pronoun/article/time-word) guards keep it origin-only and proper-noun-only; destination phrasings (to X / heading to X / arrive in X) are NEVER matched. Unit-tested 13 must-capture + 8 must-NOT-capture + 5 end-to-end block decisions, all pass; 'trip to Bar Harbor ... starting from Phoenix' captures ONLY Phoenix. The earlier 'home address in Phoenix' hole is fixed (the home-address|base anchor matches even with intervening 'your', and single-token capture avoids trailing-word/period over-capture). CHANGE 3: MESA-7 itinerary guard + MESA-8/9 prose guard now layer - itinerary turns blocked by the JSON check, confirmation/clarifying turns blocked by the prose check; MESA-7 structure untouched (+0 deletions in controllers). BLAST RADIUS: fires only for context!=='modify' AND !hasHomeOnFile AND (fabricated HOME-stop city OR prose asserts an un-typed origin). Home-on-file users, modify mode, clarifying questions (dates/party), destination mentions, and user-typed origins are all untouched; worst case is a phrasing mismatch -&gt; one extra ask (fail-safe). Client tsc+vite green; server tsc clean for the change (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). VERIFY: restart backend + fresh no-home session; destination-only prompts must yield the origin ask with NO named city and NO Build button across repeated runs, while named-origin and home-on-file flows build normally and modify mode is unaffected.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AI-MESA-10: consolidate no-home origin handling into single two-path ORIGIN RESOLUTION rule + clean copy
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -3601,6 +3601,53 @@
       <c r="I61" s="20" t="inlineStr">
         <is>
           <t>Belt-and-suspenders close of the no-home origin-fabrication category. Two prior leaks proved single-layer fixes insufficient: (i) prompt nudges (MESA-4/5/6) do not reliably stop the model naming a fabricated origin; (ii) the MESA-7 deterministic guard only inspects the &lt;itinerary&gt; JSON, so a fabricated origin stated only in PRE-ITINERARY PROSE slipped (prompt 'trip to Pittsburgh' -&gt; assistant 'Got it - starting from Columbus, Ohio', not blocked; and 'home address in Phoenix' style phrasings). NOTE: the MESA-8 prose-guard was SCOUTED earlier but never built - this task built it correctly from the start (no pre-existing extractAssertedOrigin existed on main). THREE additive changes: CHANGE 1 (PROMPT, services/ai.ts ~175-176): made the origin-naming confirmation templates EXPLICITLY CONDITIONAL and added a HARD RULE right where they are defined - the 'starting from [City, State]' and 'I'll use your home address in [CITY]' lines may be used ONLY when a real origin exists (user typed a starting city/address OR a real home is on file). When NO home on file AND no typed origin, the model is FORBIDDEN to emit any sentence naming a starting city and the ONLY permitted origin response is to ask 'Where will you be starting from?'. Placeholders only (per MESA-6 lesson); grep-verified no real city names added. No change to JSON contract / order-1 HOME instruction / noHomeDirective / hasHomeOnFile. CHANGE 2 (controllers/ai.ts): added extractAssertedOrigin(text) - an ORIGIN-ANCHORED prose scanner that returns the asserted city's first proper-noun token (single-token capture) or null, and a sibling guard block inside the existing MESA-7 no-home gate (computes its own norm/userText so the MESA-7 block is left byte-for-byte unchanged): if a no-home user's reply asserts a starting city whose first token appears in NONE of the user messages, response is replaced with NO_ORIGIN_RESPONSE. Anchors cover the scripted templates plus widened phrasings: starting from X, home address/base in|is X, your home in|is X, X as the starting point, leaving/departing (from) X, set off from X, kick off in X, launch point is X, starting point is X, begin in X. Uppercase-first-letter + stopword (pronoun/article/time-word) guards keep it origin-only and proper-noun-only; destination phrasings (to X / heading to X / arrive in X) are NEVER matched. Unit-tested 13 must-capture + 8 must-NOT-capture + 5 end-to-end block decisions, all pass; 'trip to Bar Harbor ... starting from Phoenix' captures ONLY Phoenix. The earlier 'home address in Phoenix' hole is fixed (the home-address|base anchor matches even with intervening 'your', and single-token capture avoids trailing-word/period over-capture). CHANGE 3: MESA-7 itinerary guard + MESA-8/9 prose guard now layer - itinerary turns blocked by the JSON check, confirmation/clarifying turns blocked by the prose check; MESA-7 structure untouched (+0 deletions in controllers). BLAST RADIUS: fires only for context!=='modify' AND !hasHomeOnFile AND (fabricated HOME-stop city OR prose asserts an un-typed origin). Home-on-file users, modify mode, clarifying questions (dates/party), destination mentions, and user-typed origins are all untouched; worst case is a phrasing mismatch -&gt; one extra ask (fail-safe). Client tsc+vite green; server tsc clean for the change (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). VERIFY: restart backend + fresh no-home session; destination-only prompts must yield the origin ask with NO named city and NO Build button across repeated runs, while named-origin and home-on-file flows build normally and modify mode is unaffected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="20" t="inlineStr">
+        <is>
+          <t>AI-MESA-10</t>
+        </is>
+      </c>
+      <c r="B62" s="20" t="inlineStr">
+        <is>
+          <t>Consolidate the no-home origin tangle (MESA-3/4/5/6/9 prompt rules) into ONE two-path ORIGIN RESOLUTION rule + final copy; keep MESA-7/9 deterministic guards as backstops</t>
+        </is>
+      </c>
+      <c r="C62" s="20" t="inlineStr">
+        <is>
+          <t>Cleanup/Hardening</t>
+        </is>
+      </c>
+      <c r="D62" s="20" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="E62" s="20" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="F62" s="20" t="inlineStr">
+        <is>
+          <t>DONE (06-04) - pending PROD verify</t>
+        </is>
+      </c>
+      <c r="G62" s="20" t="inlineStr">
+        <is>
+          <t>Yes - prompt consolidation + guard copy; needs backend restart + fresh no-home AND home-on-file sessions</t>
+        </is>
+      </c>
+      <c r="H62" s="20" t="inlineStr">
+        <is>
+          <t>AI-MESA-10 task 06-04</t>
+        </is>
+      </c>
+      <c r="I62" s="20" t="inlineStr">
+        <is>
+          <t>Consolidation/cleanup: replaced the entire accreted no-home origin tangle (rules from MESA-3/4/5/6/9) with ONE clean two-path ORIGIN RESOLUTION rule + final copy, and kept the deterministic guards (MESA-7 itinerary + MESA-9 prose) as backstops. WHY: six prior iterations layered overlapping prompt rules that were hard to reason about and still leaked; this collapses them to a single source of truth. PROMPT (services/ai.ts): DELETED four accreted rules (the 'Got it - starting from [City]' confirmation template, the MESA-9 HARD RULE, the static NO HOME ON FILE rule, and the HOME ON FILE 'I'll use your home address in [CITY]' template) and ADDED a single 'ORIGIN RESOLUTION - TWO PATHS, NEVER INVENT' rule: origin comes ONLY from (a) a real home on file or (b) a location the user typed in chat; never invented. Three branches with final copy: already-named -&gt; proceed no question; not-named + home-on-file -&gt; ask 'Love it - [DEST]. Starting from home, or somewhere else this trip?...'; not-named + no-home -&gt; ask '[DEST], great pick! Quick thing first - are you starting from home, or somewhere else? I don't have a home address saved to your profile yet, so if it's home, let me know your address and I'll help you save it for future trips...'. Kept rules header (173), PRECEDENCE (174), and closer (179). Shortened the long noHomeDirective body (the runtime-injected no-home signal) to a one-line reinforcement pointing at the NO-HOME path of the new rule - kept the conditional injection (hasHomeOnFile gate at line 84 + line-93 injection) because that runtime gate is what made no-home detection reliable. Line 118 HOME-stop JSON-contract instruction + startAddress: UNCHANGED (still references 'the starting-location rules above', now the new rule). [DEST] placeholder only; grep-verified no real city names added. GUARDS (controllers/ai.ts): MESA-7 itinerary guard, MESA-9 prose guard, extractAssertedOrigin, and parseItineraryBlock all BYTE-FOR-BYTE UNCHANGED (git diff shows only the NO_ORIGIN_RESPONSE constant text changed). UPDATED NO_ORIGIN_RESPONSE to a generic, [DEST]-free version of the new no-home copy (the guard can't interpolate a destination); it is now only the backstop fallback when a guard fires on a regression. Verified the new copy does NOT trip extractAssertedOrigin ('starting from home' -&gt; 'home' is a stopword -&gt; null; HOME-ON-FILE ask with a real destination -&gt; null), while a genuine fabrication still fires the backstop. SAVE PROMISE: rides the existing UX-HOME-PREFILL SaveHomeAddressModal - a no-home user who types their address in chat gets the HOME stop's startAddress, and after Build the save-home modal fires pre-filled with that address (8-field Places save). No new server hookup needed. BLAST RADIUS: no client parser depends on the old template strings (grep-confirmed); guards gated on context!=='modify' &amp;&amp; !hasHomeOnFile so home-on-file and modify mode are untouched; round-trip/[HomeCity]/campground example placeholders untouched. Client tsc+vite green; server tsc clean for the change (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). WALK-THROUGH: (a) no-home + destination-only -&gt; NO-HOME ask, names no city, no itinerary (prompt) + MESA-7/9 backstop if model regresses; (b) home-on-file + destination-only -&gt; HOME-ON-FILE ask; (c) user typed origin -&gt; proceeds, no question; (d) modify -&gt; untouched; (e) new copy never trips the prose guard. VERIFY: restart backend + fresh sessions for both no-home and home-on-file users; confirm the two-path ask copy renders and no origin is ever invented.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix SESSION-RESET-1: Cancel always starts fresh + key SessionPage per session to stop stale-state carryover
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -3648,6 +3648,53 @@
       <c r="I62" s="20" t="inlineStr">
         <is>
           <t>Consolidation/cleanup: replaced the entire accreted no-home origin tangle (rules from MESA-3/4/5/6/9) with ONE clean two-path ORIGIN RESOLUTION rule + final copy, and kept the deterministic guards (MESA-7 itinerary + MESA-9 prose) as backstops. WHY: six prior iterations layered overlapping prompt rules that were hard to reason about and still leaked; this collapses them to a single source of truth. PROMPT (services/ai.ts): DELETED four accreted rules (the 'Got it - starting from [City]' confirmation template, the MESA-9 HARD RULE, the static NO HOME ON FILE rule, and the HOME ON FILE 'I'll use your home address in [CITY]' template) and ADDED a single 'ORIGIN RESOLUTION - TWO PATHS, NEVER INVENT' rule: origin comes ONLY from (a) a real home on file or (b) a location the user typed in chat; never invented. Three branches with final copy: already-named -&gt; proceed no question; not-named + home-on-file -&gt; ask 'Love it - [DEST]. Starting from home, or somewhere else this trip?...'; not-named + no-home -&gt; ask '[DEST], great pick! Quick thing first - are you starting from home, or somewhere else? I don't have a home address saved to your profile yet, so if it's home, let me know your address and I'll help you save it for future trips...'. Kept rules header (173), PRECEDENCE (174), and closer (179). Shortened the long noHomeDirective body (the runtime-injected no-home signal) to a one-line reinforcement pointing at the NO-HOME path of the new rule - kept the conditional injection (hasHomeOnFile gate at line 84 + line-93 injection) because that runtime gate is what made no-home detection reliable. Line 118 HOME-stop JSON-contract instruction + startAddress: UNCHANGED (still references 'the starting-location rules above', now the new rule). [DEST] placeholder only; grep-verified no real city names added. GUARDS (controllers/ai.ts): MESA-7 itinerary guard, MESA-9 prose guard, extractAssertedOrigin, and parseItineraryBlock all BYTE-FOR-BYTE UNCHANGED (git diff shows only the NO_ORIGIN_RESPONSE constant text changed). UPDATED NO_ORIGIN_RESPONSE to a generic, [DEST]-free version of the new no-home copy (the guard can't interpolate a destination); it is now only the backstop fallback when a guard fires on a regression. Verified the new copy does NOT trip extractAssertedOrigin ('starting from home' -&gt; 'home' is a stopword -&gt; null; HOME-ON-FILE ask with a real destination -&gt; null), while a genuine fabrication still fires the backstop. SAVE PROMISE: rides the existing UX-HOME-PREFILL SaveHomeAddressModal - a no-home user who types their address in chat gets the HOME stop's startAddress, and after Build the save-home modal fires pre-filled with that address (8-field Places save). No new server hookup needed. BLAST RADIUS: no client parser depends on the old template strings (grep-confirmed); guards gated on context!=='modify' &amp;&amp; !hasHomeOnFile so home-on-file and modify mode are untouched; round-trip/[HomeCity]/campground example placeholders untouched. Client tsc+vite green; server tsc clean for the change (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). WALK-THROUGH: (a) no-home + destination-only -&gt; NO-HOME ask, names no city, no itinerary (prompt) + MESA-7/9 backstop if model regresses; (b) home-on-file + destination-only -&gt; HOME-ON-FILE ask; (c) user typed origin -&gt; proceeds, no question; (d) modify -&gt; untouched; (e) new copy never trips the prose guard. VERIFY: restart backend + fresh sessions for both no-home and home-on-file users; confirm the two-path ask copy renders and no origin is ever invented.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="20" t="inlineStr">
+        <is>
+          <t>SESSION-RESET-1</t>
+        </is>
+      </c>
+      <c r="B63" s="20" t="inlineStr">
+        <is>
+          <t>'Cancel this plan' then new plan (no refresh) ~50% silently resumes a stale sibling session; contaminated context -&gt; off-topic refusal (hard refresh fixes it)</t>
+        </is>
+      </c>
+      <c r="C63" s="20" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="D63" s="20" t="inlineStr">
+        <is>
+          <t>Frontend/Sessions</t>
+        </is>
+      </c>
+      <c r="E63" s="20" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="F63" s="20" t="inlineStr">
+        <is>
+          <t>DONE (06-04) - pending PROD verify</t>
+        </is>
+      </c>
+      <c r="G63" s="20" t="inlineStr">
+        <is>
+          <t>Yes - frontend session-state reset; verify in browser</t>
+        </is>
+      </c>
+      <c r="H63" s="20" t="inlineStr">
+        <is>
+          <t>SESSION-RESET-1 task 06-04 (scout + fix)</t>
+        </is>
+      </c>
+      <c r="I63" s="20" t="inlineStr">
+        <is>
+          <t>Frontend stale-state bug. REPRO: start a plan, click 'Cancel this plan', then start a NEW plan in the same page (no refresh) -&gt; ~50% of the time the assistant returns the off-topic refusal ('I'm RoamReady's trip planning assistant...'); a hard refresh always fixes it. NOT a backend/prompt bug (same commit works after refresh). ROOT CAUSE (two compounding defects): (1) handleCancel navigated to /sessions/new, which runs SessionNewPage's silent-resume heuristics: Check A (lastVisitedSessionId match) AND Check B (session updatedAt &lt; 5 min ago). Cancel cleared the Check-A flag but NOT Check B, so Check B could latch onto a stale SIBLING PLANNING session (these accumulate - 'New trip'/createFresh leave prior sessions in PLANNING; getLatestActive returns any PLANNING session that has messages regardless of age) and silently RESUME it instead of starting fresh. The resumed session's old conversation hydrated into SessionPage and the user's next message was appended to it and sent to /ai/chat -&gt; the model saw a stale/off-topic-ending conversation and returned the off-topic refusal. ~50% = depends on whether a recent (&lt;5min) PLANNING+messages sibling exists. (2) The /sessions/:id route rendered &lt;SessionPage/&gt; with NO key, so React reused the same instance across session switches (param-only change, no unmount), carrying in-memory messages/itinerary plus the 1.5s autosave hook into the next session until the async [sessionId] hydrate reset them - a window the autosave (write old messages to new sessionId) and the next send could race. A hard refresh fixed it because it fully remounts and re-hydrates from the server row and bypasses the resume heuristics. FIX (frontend only; no backend/prompt/guard/persisted-data change): FIX 1 (client/src/pages/SessionPage.tsx handleCancel): an explicit Cancel no longer routes through /sessions/new; it now deletes the current session, clears lastVisitedSessionId, CREATES a brand-new empty session directly (mirroring handleNewTrip) and navigates straight to it - so Cancel ALWAYS lands in a fresh empty session, never a resumed sibling. Kept the isProcessing guard + error handling. FIX 2 (client/src/App.tsx): wrapped the /sessions/:id route in KeyedSessionPage which reads useParams().id and renders &lt;SessionPage key={id} /&gt;, forcing unmount-&gt;remount with fresh state on every session switch (same clean slate as a refresh), eliminating the cross-session in-memory carryover and the autosave-to-wrong-session race. BLAST RADIUS: Fix 1 changes ONLY explicit Cancel (always fresh - desired); ordinary in-app silent-resume (Profile -&gt; back to a session) is UNCHANGED (still uses SessionNewPage Check A/B). Fix 2's key remount is standard for param-routed detail pages; cost is a re-hydrate on session switch (already happened via the effect). WALK-THROUGH: (a) Cancel-&gt;new = fresh empty session, no stale messages sent; (b) switching between two trips = each remounts clean, no carryover; (c) Profile-&gt;back = still resumes (Check A/B intact); (d) New trip button = fresh session, prior session left PLANNING as before. Client tsc+vite green; server tsc clean (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). VERIFY: on a fresh load, plan -&gt; Cancel -&gt; plan again repeatedly with NO refresh; must never get the off-topic refusal and must always start empty.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix SCOPE-1: add positive in-scope anchor so casual trip phrasings aren't refused as off-topic
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
+++ b/documents/Backlog Tracker/RoamReady_Bug_Todo_Tracker_2026-06-04.xlsx
@@ -723,7 +723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="20" min="1" max="1"/>
@@ -3695,6 +3695,53 @@
       <c r="I63" s="20" t="inlineStr">
         <is>
           <t>Frontend stale-state bug. REPRO: start a plan, click 'Cancel this plan', then start a NEW plan in the same page (no refresh) -&gt; ~50% of the time the assistant returns the off-topic refusal ('I'm RoamReady's trip planning assistant...'); a hard refresh always fixes it. NOT a backend/prompt bug (same commit works after refresh). ROOT CAUSE (two compounding defects): (1) handleCancel navigated to /sessions/new, which runs SessionNewPage's silent-resume heuristics: Check A (lastVisitedSessionId match) AND Check B (session updatedAt &lt; 5 min ago). Cancel cleared the Check-A flag but NOT Check B, so Check B could latch onto a stale SIBLING PLANNING session (these accumulate - 'New trip'/createFresh leave prior sessions in PLANNING; getLatestActive returns any PLANNING session that has messages regardless of age) and silently RESUME it instead of starting fresh. The resumed session's old conversation hydrated into SessionPage and the user's next message was appended to it and sent to /ai/chat -&gt; the model saw a stale/off-topic-ending conversation and returned the off-topic refusal. ~50% = depends on whether a recent (&lt;5min) PLANNING+messages sibling exists. (2) The /sessions/:id route rendered &lt;SessionPage/&gt; with NO key, so React reused the same instance across session switches (param-only change, no unmount), carrying in-memory messages/itinerary plus the 1.5s autosave hook into the next session until the async [sessionId] hydrate reset them - a window the autosave (write old messages to new sessionId) and the next send could race. A hard refresh fixed it because it fully remounts and re-hydrates from the server row and bypasses the resume heuristics. FIX (frontend only; no backend/prompt/guard/persisted-data change): FIX 1 (client/src/pages/SessionPage.tsx handleCancel): an explicit Cancel no longer routes through /sessions/new; it now deletes the current session, clears lastVisitedSessionId, CREATES a brand-new empty session directly (mirroring handleNewTrip) and navigates straight to it - so Cancel ALWAYS lands in a fresh empty session, never a resumed sibling. Kept the isProcessing guard + error handling. FIX 2 (client/src/App.tsx): wrapped the /sessions/:id route in KeyedSessionPage which reads useParams().id and renders &lt;SessionPage key={id} /&gt;, forcing unmount-&gt;remount with fresh state on every session switch (same clean slate as a refresh), eliminating the cross-session in-memory carryover and the autosave-to-wrong-session race. BLAST RADIUS: Fix 1 changes ONLY explicit Cancel (always fresh - desired); ordinary in-app silent-resume (Profile -&gt; back to a session) is UNCHANGED (still uses SessionNewPage Check A/B). Fix 2's key remount is standard for param-routed detail pages; cost is a re-hydrate on session switch (already happened via the effect). WALK-THROUGH: (a) Cancel-&gt;new = fresh empty session, no stale messages sent; (b) switching between two trips = each remounts clean, no carryover; (c) Profile-&gt;back = still resumes (Check A/B intact); (d) New trip button = fresh session, prior session left PLANNING as before. Client tsc+vite green; server tsc clean (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). VERIFY: on a fresh load, plan -&gt; Cancel -&gt; plan again repeatedly with NO refresh; must never get the off-topic refusal and must always start empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="20" t="inlineStr">
+        <is>
+          <t>SCOPE-1</t>
+        </is>
+      </c>
+      <c r="B64" s="20" t="inlineStr">
+        <is>
+          <t>Off-topic scope guardrail over-fires on casually-phrased valid trip requests ('Show me around X', 'Send me to X') - negative-only classifier with no positive trip-intent definition</t>
+        </is>
+      </c>
+      <c r="C64" s="20" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="D64" s="20" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="E64" s="20" t="inlineStr">
+        <is>
+          <t>P1 - High</t>
+        </is>
+      </c>
+      <c r="F64" s="20" t="inlineStr">
+        <is>
+          <t>DONE (06-04) - pending PROD verify</t>
+        </is>
+      </c>
+      <c r="G64" s="20" t="inlineStr">
+        <is>
+          <t>Yes - prompt-only; needs backend restart + fresh session</t>
+        </is>
+      </c>
+      <c r="H64" s="20" t="inlineStr">
+        <is>
+          <t>SCOPE-1 task 06-04 (scout + fix)</t>
+        </is>
+      </c>
+      <c r="I64" s="20" t="inlineStr">
+        <is>
+          <t>Scope guardrail over-fires on casually-phrased but VALID trip requests. REPRO: 'Show me around Taos, New Mexico' and 'Send me to Galveston, Texas' triggered the off-topic refusal ('I'm RoamReady's trip planning assistant and I can only help with outdoor travel planning...') instead of proceeding to the origin question (Taos sometimes half-recovered, Galveston dead-ended) - unambiguous trip intents wrongly declined. ROOT CAUSE: the scope/off-topic rule (services/ai.ts line 91) is NEGATIVE-ONLY - it enumerates off-topic categories and says 'refuse ANYTHING unrelated... under any circumstances' but has NO positive definition of a valid trip request. The prompt's recognized trip-request signals are keyed on plan/create/trip-to/going-to/from-X-to-Y phrasings (Surprise-rule PRECEDENCE line 106 + pervasive 'plan a trip' examples), so casual phrasings with no trip keyword ('show me around X', 'send me to X', 'take me to X') match no positive pattern and fall through to the firm refusal; 'show me around' can even read as a general-info request (caught by 'general knowledge questions'). The half-recover-vs-dead-end inconsistency is classic ambiguous-classification nondeterminism. Scope is evaluated FIRST (line 91, before NAMED DESTINATION ~115 and ORIGIN RESOLUTION ~175-179), so a misfire never reaches origin resolution - the new MESA-10 rule neither causes nor can rescue it. FIX (prompt-only, additive, +3/-1 in services/ai.ts; did NOT delete the refusal rule, NAMED DESTINATION RULE, ORIGIN RESOLUTION, MESA guards, or JSON contract): added a positive IN-SCOPE anchor immediately after the refusal rule - 'A WISH TO GO somewhere is ALWAYS a trip request': any message naming a place/region/park/landmark the user wants to go to or be shown around, in ANY casual phrasing (show me around [Place], send me to [Place], take me to [Place], get me to [Place], I want to go to [Place], let's visit [Place], how about [Place]?, [Place] sounds fun, or just naming [Place]) is a VALID trip request -&gt; proceed to trip planning (origin/ORIGIN RESOLUTION step), NEVER refuse. The refusal now applies ONLY to messages with NO travel intent (poem, coding, medical/legal/financial advice, current events, other non-travel). Added an ambiguity TIEBREAKER: when ambiguous between off-topic and a casual trip request, ALWAYS assume trip request. Also softened line 91's absolute 'under any circumstances' with a parenthetical deferral to the IN-SCOPE rule. Placeholders only ([Place]); grep-verified no real city names added. Client tsc+vite green; server tsc clean (pre-existing redis.ts/prisma.ts TS2742 junction artifacts only). WALK-THROUGH: (a) 'Send me to Galveston' -&gt; in-scope -&gt; origin question, no refusal; (b) 'Show me around Taos' -&gt; in-scope -&gt; proceeds; (c) 'Plan a trip to X' -&gt; still works; (d) 'write me a poem' / 'what's the weather in general' -&gt; STILL refused (no travel intent); (e) ambiguous -&gt; defaults to trip request. VERIFY: restart backend + fresh session; casual destination phrasings must proceed to the origin question, genuine off-topic must still get the refusal.</t>
         </is>
       </c>
     </row>

</xml_diff>